<commit_message>
Atualização de alguns erros e lentidão nos formulários
</commit_message>
<xml_diff>
--- a/includes/fin_empenhos/planilha_modelo_empenhos.xlsx
+++ b/includes/fin_empenhos/planilha_modelo_empenhos.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp2\htdocs\gceemv2\includes\fin_empenhos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp2\htdocs\ambiente_trabalho\gceem\includes\fin_empenhos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E80C617F-70A1-4D05-9336-638FF5544300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A13496-A419-4D79-ABE6-D58E0E19EC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10245" yWindow="0" windowWidth="10245" windowHeight="10920" xr2:uid="{401957C4-9E45-4D03-92D2-E99DBBD38077}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{401957C4-9E45-4D03-92D2-E99DBBD38077}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,58 +27,58 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
-    <t>Cnpj_Fornecedor</t>
-  </si>
-  <si>
-    <t>requisitante</t>
-  </si>
-  <si>
-    <t>destinatario</t>
-  </si>
-  <si>
-    <t>nota_credito</t>
-  </si>
-  <si>
-    <t>plano_interno</t>
-  </si>
-  <si>
-    <t>natureza_despesa</t>
-  </si>
-  <si>
-    <t>item_oog</t>
-  </si>
-  <si>
-    <t>finalidade</t>
-  </si>
-  <si>
-    <t>tipo_empenho</t>
-  </si>
-  <si>
-    <t>necessidade_contrato</t>
-  </si>
-  <si>
-    <t>data_empenho</t>
-  </si>
-  <si>
-    <t>nmr_empenho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obra </t>
-  </si>
-  <si>
-    <t>ano</t>
-  </si>
-  <si>
-    <t>categoria do empenho (Peças, serviços, lubrificantes)</t>
-  </si>
-  <si>
     <t>Local do Empenho</t>
   </si>
   <si>
     <t>resto_pagar (sim ou não)</t>
   </si>
   <si>
-    <t xml:space="preserve">valor_empenhado </t>
+    <t>Marca do empenho</t>
+  </si>
+  <si>
+    <t>CNPJ do fornecedor</t>
+  </si>
+  <si>
+    <t>Requisitante (Cmt Ceem)</t>
+  </si>
+  <si>
+    <t>Destinatario Req (S4/FISC ADM)</t>
+  </si>
+  <si>
+    <t>Nota de Crédito</t>
+  </si>
+  <si>
+    <t>Plano Interno</t>
+  </si>
+  <si>
+    <t>Natureza da Despesa</t>
+  </si>
+  <si>
+    <t>Item OOG (SIOC)</t>
+  </si>
+  <si>
+    <t>Finalidade (peças, serviços, lubrificantes e etc)</t>
+  </si>
+  <si>
+    <t>Tipo empenho  (global, ordinário e etc)</t>
+  </si>
+  <si>
+    <t>Necessidade de contrato (sim ou não)</t>
+  </si>
+  <si>
+    <t>Data empenho</t>
+  </si>
+  <si>
+    <t>Nmr do empenho</t>
+  </si>
+  <si>
+    <t>Obra</t>
+  </si>
+  <si>
+    <t>Ano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor empenhado </t>
   </si>
 </sst>
 </file>
@@ -114,13 +114,83 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="20">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -133,10 +203,37 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E59AC37D-6C22-497C-B68B-6623965A4E14}" name="Tabela1" displayName="Tabela1" ref="A1:R16" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:R16" xr:uid="{E59AC37D-6C22-497C-B68B-6623965A4E14}"/>
+  <tableColumns count="18">
+    <tableColumn id="1" xr3:uid="{8613D4DE-1DFE-4D1C-8E8E-E44FB1AC8E28}" name="CNPJ do fornecedor" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{88ED2915-4638-4D81-8DCC-5F9A7C018C6F}" name="Requisitante (Cmt Ceem)" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{E49D4C95-C8BE-4F99-B3AA-F1FF9F82668C}" name="Destinatario Req (S4/FISC ADM)" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{AE05294B-EDC3-4684-AB85-CA121F0D1A12}" name="Nota de Crédito" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{33487E38-7853-4FEC-AC7B-1E6DADE71AEE}" name="Plano Interno" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{7C5743F7-EDBF-40BF-8C0B-B5BA2BE532E4}" name="Natureza da Despesa" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{F584DAB0-89F9-449A-AE6E-593AD62D4A46}" name="Item OOG (SIOC)" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{09A5DD74-53BE-4AAE-B2CB-8EC8612C983D}" name="Finalidade (peças, serviços, lubrificantes e etc)" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{E0296721-141F-4951-A94F-89A4919B4057}" name="Tipo empenho  (global, ordinário e etc)" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{4EF75650-005E-4ECE-A408-8F292B24B49D}" name="Necessidade de contrato (sim ou não)" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{90709405-CB83-478F-B7E2-459BFEBB0E97}" name="Data empenho" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{EEAB629E-0D17-44C7-88BE-AE6C8CC0C364}" name="Nmr do empenho" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{74AE2F33-DD6E-4399-BB5C-20F93D73D202}" name="Obra" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{B44792B3-80EF-492C-8D8A-EE6CCF1BB08E}" name="Ano" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{B652AB87-D74C-403A-9347-C249AC194A80}" name="Marca do empenho" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{F62FEB86-C9E7-4C79-9339-9EC00776B5BB}" name="Local do Empenho" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{3F83AF95-EC08-48A2-9CF5-2A0A1A71E736}" name="resto_pagar (sim ou não)" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{E84F1681-97DD-4B18-AF88-7015B3290E8F}" name="Valor empenhado " dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -174,7 +271,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -280,7 +377,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -422,7 +519,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -430,84 +527,387 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9560EDC9-EBB5-4266-BDDE-0C3A9F35F0C3}">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" customWidth="1"/>
     <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
-    <col min="9" max="9" width="17.5703125" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" customWidth="1"/>
-    <col min="11" max="11" width="15.28515625" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" customWidth="1"/>
+    <col min="8" max="8" width="36.42578125" customWidth="1"/>
+    <col min="9" max="9" width="31.85546875" customWidth="1"/>
+    <col min="10" max="10" width="26" customWidth="1"/>
+    <col min="11" max="11" width="17.42578125" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" customWidth="1"/>
     <col min="15" max="15" width="49.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="23.140625" customWidth="1"/>
-    <col min="18" max="18" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.140625" customWidth="1"/>
+    <col min="17" max="17" width="25" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="Q1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>